<commit_message>
feat: Arrumando organizacao do projeto
</commit_message>
<xml_diff>
--- a/Execelteste/Base.xlsx
+++ b/Execelteste/Base.xlsx
@@ -27,18 +27,18 @@
     <t>Numero</t>
   </si>
   <si>
+    <t>Email Insper</t>
+  </si>
+  <si>
+    <t>Email Pessoal</t>
+  </si>
+  <si>
     <t>Semestre</t>
   </si>
   <si>
     <t>Curso</t>
   </si>
   <si>
-    <t>Email Insper</t>
-  </si>
-  <si>
-    <t>Email Pessoal</t>
-  </si>
-  <si>
     <t>Primeira Opção</t>
   </si>
   <si>
@@ -54,15 +54,15 @@
     <t>Teste 1</t>
   </si>
   <si>
+    <t>teste1@al.insper.edu.br</t>
+  </si>
+  <si>
+    <t>teste1@exemplo.com</t>
+  </si>
+  <si>
     <t>Engenharia</t>
   </si>
   <si>
-    <t>teste1@al.insper.edu.br</t>
-  </si>
-  <si>
-    <t>teste1@exemplo.com</t>
-  </si>
-  <si>
     <t>quarta</t>
   </si>
   <si>
@@ -72,43 +72,43 @@
     <t>Teste 2</t>
   </si>
   <si>
+    <t>teste2@al.insper.edu.br</t>
+  </si>
+  <si>
+    <t>teste2@exemplo.com</t>
+  </si>
+  <si>
     <t>Direito</t>
   </si>
   <si>
-    <t>teste2@al.insper.edu.br</t>
-  </si>
-  <si>
-    <t>teste2@exemplo.com</t>
-  </si>
-  <si>
     <t>segunda</t>
   </si>
   <si>
     <t>Teste 3</t>
   </si>
   <si>
+    <t>teste3@al.insper.edu.br</t>
+  </si>
+  <si>
+    <t>teste3@exemplo.com</t>
+  </si>
+  <si>
     <t>ADM</t>
   </si>
   <si>
-    <t>teste3@al.insper.edu.br</t>
-  </si>
-  <si>
-    <t>teste3@exemplo.com</t>
-  </si>
-  <si>
     <t>terca</t>
   </si>
   <si>
     <t>Teste 4</t>
   </si>
   <si>
+    <t>teste4@al.insper.edu.br</t>
+  </si>
+  <si>
+    <t>teste4@exemplo.com</t>
+  </si>
+  <si>
     <t>Econo</t>
-  </si>
-  <si>
-    <t>teste4@al.insper.edu.br</t>
-  </si>
-  <si>
-    <t>teste4@exemplo.com</t>
   </si>
   <si>
     <t>Teste 5</t>
@@ -1439,7 +1439,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="E52:E108" displayName="Table_3" name="Table_3" id="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="G52:G108" displayName="Table_3" name="Table_3" id="3">
   <tableColumns count="1">
     <tableColumn name="Column1" id="1"/>
   </tableColumns>
@@ -1662,9 +1662,9 @@
     <col customWidth="1" min="2" max="2" width="8.88"/>
     <col customWidth="1" min="3" max="3" width="12.0"/>
     <col customWidth="1" min="4" max="4" width="10.0"/>
-    <col customWidth="1" min="5" max="5" width="8.63"/>
-    <col customWidth="1" min="6" max="6" width="10.38"/>
-    <col customWidth="1" min="7" max="8" width="22.63"/>
+    <col customWidth="1" min="5" max="6" width="22.63"/>
+    <col customWidth="1" min="7" max="7" width="8.63"/>
+    <col customWidth="1" min="8" max="8" width="10.38"/>
     <col customWidth="1" min="9" max="9" width="13.88"/>
     <col customWidth="1" min="10" max="10" width="14.25"/>
     <col customWidth="1" min="11" max="11" width="13.75"/>
@@ -1722,14 +1722,14 @@
       <c r="D2" s="5">
         <v>9.99999999E8</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="5">
         <v>1.0</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>14</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>15</v>
@@ -1757,14 +1757,14 @@
         <f t="shared" ref="D3:D108" si="1">D2-1</f>
         <v>999999998</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="5">
         <v>2.0</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>21</v>
@@ -1790,14 +1790,14 @@
         <f t="shared" si="1"/>
         <v>999999997</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="5">
         <v>3.0</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>25</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>26</v>
@@ -1829,14 +1829,14 @@
         <f t="shared" si="1"/>
         <v>999999996</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="5">
         <v>1.0</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>31</v>
@@ -1866,17 +1866,17 @@
         <f t="shared" si="1"/>
         <v>999999995</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="5">
         <v>2.0</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>33</v>
-      </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>22</v>
@@ -1899,17 +1899,17 @@
         <f t="shared" si="1"/>
         <v>999999994</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="5">
         <v>3.0</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>36</v>
+      <c r="H7" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>17</v>
@@ -1938,17 +1938,17 @@
         <f t="shared" si="1"/>
         <v>999999993</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="5">
         <v>1.0</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>38</v>
+      <c r="H8" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>22</v>
@@ -1977,17 +1977,17 @@
         <f t="shared" si="1"/>
         <v>999999992</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" s="5">
         <v>2.0</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>40</v>
+      <c r="H9" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>16</v>
@@ -2014,17 +2014,17 @@
         <f t="shared" si="1"/>
         <v>999999991</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" s="5">
         <v>3.0</v>
       </c>
-      <c r="F10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>42</v>
+      <c r="H10" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>27</v>
@@ -2051,17 +2051,17 @@
         <f t="shared" si="1"/>
         <v>999999990</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="G11" s="5">
         <v>1.0</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>44</v>
+      <c r="H11" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>17</v>
@@ -2084,17 +2084,17 @@
         <f t="shared" si="1"/>
         <v>999999989</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="5">
         <v>2.0</v>
       </c>
-      <c r="F12" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>46</v>
+      <c r="H12" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>16</v>
@@ -2123,17 +2123,17 @@
         <f t="shared" si="1"/>
         <v>999999988</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G13" s="5">
         <v>3.0</v>
       </c>
-      <c r="F13" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>48</v>
+      <c r="H13" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>27</v>
@@ -2156,17 +2156,17 @@
         <f t="shared" si="1"/>
         <v>999999987</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" s="5">
         <v>1.0</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>50</v>
+      <c r="H14" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>27</v>
@@ -2195,17 +2195,17 @@
         <f t="shared" si="1"/>
         <v>999999986</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" s="5">
         <v>2.0</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>52</v>
+      <c r="H15" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>22</v>
@@ -2228,17 +2228,17 @@
         <f t="shared" si="1"/>
         <v>999999985</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G16" s="5">
         <v>3.0</v>
       </c>
-      <c r="F16" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>54</v>
+      <c r="H16" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>17</v>
@@ -2267,17 +2267,17 @@
         <f t="shared" si="1"/>
         <v>999999984</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G17" s="5">
         <v>1.0</v>
       </c>
-      <c r="F17" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>56</v>
+      <c r="H17" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>16</v>
@@ -2304,17 +2304,17 @@
         <f t="shared" si="1"/>
         <v>999999983</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G18" s="5">
         <v>2.0</v>
       </c>
-      <c r="F18" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>58</v>
+      <c r="H18" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>22</v>
@@ -2339,17 +2339,17 @@
         <f t="shared" si="1"/>
         <v>999999982</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" s="5">
         <v>3.0</v>
       </c>
-      <c r="F19" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="H19" s="7" t="s">
-        <v>60</v>
+      <c r="H19" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>16</v>
@@ -2376,17 +2376,17 @@
         <f t="shared" si="1"/>
         <v>999999981</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G20" s="5">
         <v>1.0</v>
       </c>
-      <c r="F20" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>62</v>
+      <c r="H20" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>22</v>
@@ -2415,17 +2415,17 @@
         <f t="shared" si="1"/>
         <v>999999980</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G21" s="5">
         <v>2.0</v>
       </c>
-      <c r="F21" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="H21" s="7" t="s">
-        <v>64</v>
+      <c r="H21" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>22</v>
@@ -2448,17 +2448,17 @@
         <f t="shared" si="1"/>
         <v>999999979</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G22" s="5">
         <v>3.0</v>
       </c>
-      <c r="F22" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="H22" s="7" t="s">
-        <v>66</v>
+      <c r="H22" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>27</v>
@@ -2485,17 +2485,17 @@
         <f t="shared" si="1"/>
         <v>999999978</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G23" s="5">
         <v>1.0</v>
       </c>
-      <c r="F23" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>68</v>
+      <c r="H23" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>16</v>
@@ -2522,17 +2522,17 @@
         <f t="shared" si="1"/>
         <v>999999977</v>
       </c>
-      <c r="E24" s="5">
+      <c r="E24" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="G24" s="5">
         <v>2.0</v>
       </c>
-      <c r="F24" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>70</v>
+      <c r="H24" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>22</v>
@@ -2559,17 +2559,17 @@
         <f t="shared" si="1"/>
         <v>999999976</v>
       </c>
-      <c r="E25" s="5">
+      <c r="E25" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G25" s="5">
         <v>3.0</v>
       </c>
-      <c r="F25" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>72</v>
+      <c r="H25" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>17</v>
@@ -2596,17 +2596,17 @@
         <f t="shared" si="1"/>
         <v>999999975</v>
       </c>
-      <c r="E26" s="5">
+      <c r="E26" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G26" s="5">
         <v>1.0</v>
       </c>
-      <c r="F26" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>74</v>
+      <c r="H26" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>16</v>
@@ -2633,17 +2633,17 @@
         <f t="shared" si="1"/>
         <v>999999974</v>
       </c>
-      <c r="E27" s="5">
+      <c r="E27" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="G27" s="5">
         <v>2.0</v>
       </c>
-      <c r="F27" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>76</v>
+      <c r="H27" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>27</v>
@@ -2672,17 +2672,17 @@
         <f t="shared" si="1"/>
         <v>999999973</v>
       </c>
-      <c r="E28" s="5">
+      <c r="E28" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="G28" s="5">
         <v>3.0</v>
       </c>
-      <c r="F28" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="H28" s="7" t="s">
-        <v>78</v>
+      <c r="H28" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>16</v>
@@ -2705,17 +2705,17 @@
         <f t="shared" si="1"/>
         <v>999999972</v>
       </c>
-      <c r="E29" s="5">
+      <c r="E29" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="G29" s="5">
         <v>1.0</v>
       </c>
-      <c r="F29" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>80</v>
+      <c r="H29" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>16</v>
@@ -2744,17 +2744,17 @@
         <f t="shared" si="1"/>
         <v>999999971</v>
       </c>
-      <c r="E30" s="5">
+      <c r="E30" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="G30" s="5">
         <v>2.0</v>
       </c>
-      <c r="F30" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>82</v>
+      <c r="H30" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>16</v>
@@ -2781,17 +2781,17 @@
         <f t="shared" si="1"/>
         <v>999999970</v>
       </c>
-      <c r="E31" s="5">
+      <c r="E31" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="G31" s="5">
         <v>3.0</v>
       </c>
-      <c r="F31" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>84</v>
+      <c r="H31" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>22</v>
@@ -2818,17 +2818,17 @@
         <f t="shared" si="1"/>
         <v>999999969</v>
       </c>
-      <c r="E32" s="5">
+      <c r="E32" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="G32" s="5">
         <v>1.0</v>
       </c>
-      <c r="F32" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>86</v>
+      <c r="H32" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>16</v>
@@ -2857,17 +2857,17 @@
         <f t="shared" si="1"/>
         <v>999999968</v>
       </c>
-      <c r="E33" s="5">
+      <c r="E33" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G33" s="5">
         <v>2.0</v>
       </c>
-      <c r="F33" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="H33" s="7" t="s">
-        <v>88</v>
+      <c r="H33" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>16</v>
@@ -2896,17 +2896,17 @@
         <f t="shared" si="1"/>
         <v>999999967</v>
       </c>
-      <c r="E34" s="5">
+      <c r="E34" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="G34" s="5">
         <v>3.0</v>
       </c>
-      <c r="F34" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="H34" s="7" t="s">
-        <v>90</v>
+      <c r="H34" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>22</v>
@@ -2929,17 +2929,17 @@
         <f t="shared" si="1"/>
         <v>999999966</v>
       </c>
-      <c r="E35" s="5">
+      <c r="E35" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G35" s="5">
         <v>1.0</v>
       </c>
-      <c r="F35" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G35" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="H35" s="7" t="s">
-        <v>92</v>
+      <c r="H35" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I35" s="5" t="s">
         <v>17</v>
@@ -2968,17 +2968,17 @@
         <f t="shared" si="1"/>
         <v>999999965</v>
       </c>
-      <c r="E36" s="5">
+      <c r="E36" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G36" s="5">
         <v>2.0</v>
       </c>
-      <c r="F36" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="H36" s="7" t="s">
-        <v>94</v>
+      <c r="H36" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="I36" s="5" t="s">
         <v>22</v>
@@ -3001,17 +3001,17 @@
         <f t="shared" si="1"/>
         <v>999999964</v>
       </c>
-      <c r="E37" s="5">
+      <c r="E37" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G37" s="5">
         <v>3.0</v>
       </c>
-      <c r="F37" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G37" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="H37" s="7" t="s">
-        <v>96</v>
+      <c r="H37" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="I37" s="5" t="s">
         <v>22</v>
@@ -3040,17 +3040,17 @@
         <f t="shared" si="1"/>
         <v>999999963</v>
       </c>
-      <c r="E38" s="5">
+      <c r="E38" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G38" s="5">
         <v>1.0</v>
       </c>
-      <c r="F38" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G38" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>98</v>
+      <c r="H38" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="I38" s="5" t="s">
         <v>22</v>
@@ -3079,17 +3079,17 @@
         <f t="shared" si="1"/>
         <v>999999962</v>
       </c>
-      <c r="E39" s="5">
+      <c r="E39" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="G39" s="5">
         <v>2.0</v>
       </c>
-      <c r="F39" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>100</v>
+      <c r="H39" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>22</v>
@@ -3118,17 +3118,17 @@
         <f t="shared" si="1"/>
         <v>999999961</v>
       </c>
-      <c r="E40" s="5">
+      <c r="E40" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G40" s="5">
         <v>3.0</v>
       </c>
-      <c r="F40" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G40" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="H40" s="7" t="s">
-        <v>102</v>
+      <c r="H40" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="I40" s="5" t="s">
         <v>22</v>
@@ -3157,17 +3157,17 @@
         <f t="shared" si="1"/>
         <v>999999960</v>
       </c>
-      <c r="E41" s="5">
+      <c r="E41" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="G41" s="5">
         <v>1.0</v>
       </c>
-      <c r="F41" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G41" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="H41" s="7" t="s">
-        <v>104</v>
+      <c r="H41" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="I41" s="5" t="s">
         <v>16</v>
@@ -3196,17 +3196,17 @@
         <f t="shared" si="1"/>
         <v>999999959</v>
       </c>
-      <c r="E42" s="5">
+      <c r="E42" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="G42" s="5">
         <v>2.0</v>
       </c>
-      <c r="F42" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="H42" s="7" t="s">
-        <v>106</v>
+      <c r="H42" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="I42" s="5" t="s">
         <v>16</v>
@@ -3235,17 +3235,17 @@
         <f t="shared" si="1"/>
         <v>999999958</v>
       </c>
-      <c r="E43" s="5">
+      <c r="E43" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="G43" s="5">
         <v>3.0</v>
       </c>
-      <c r="F43" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G43" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="H43" s="7" t="s">
-        <v>108</v>
+      <c r="H43" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I43" s="5" t="s">
         <v>16</v>
@@ -3274,17 +3274,17 @@
         <f t="shared" si="1"/>
         <v>999999957</v>
       </c>
-      <c r="E44" s="5">
+      <c r="E44" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="G44" s="5">
         <v>1.0</v>
       </c>
-      <c r="F44" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G44" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="H44" s="7" t="s">
-        <v>110</v>
+      <c r="H44" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>16</v>
@@ -3311,17 +3311,17 @@
         <f t="shared" si="1"/>
         <v>999999956</v>
       </c>
-      <c r="E45" s="5">
+      <c r="E45" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="G45" s="5">
         <v>2.0</v>
       </c>
-      <c r="F45" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G45" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>112</v>
+      <c r="H45" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>22</v>
@@ -3348,17 +3348,17 @@
         <f t="shared" si="1"/>
         <v>999999955</v>
       </c>
-      <c r="E46" s="5">
+      <c r="E46" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="G46" s="5">
         <v>3.0</v>
       </c>
-      <c r="F46" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G46" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="H46" s="7" t="s">
-        <v>114</v>
+      <c r="H46" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="I46" s="5" t="s">
         <v>16</v>
@@ -3385,17 +3385,17 @@
         <f t="shared" si="1"/>
         <v>999999954</v>
       </c>
-      <c r="E47" s="5">
+      <c r="E47" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="G47" s="5">
         <v>1.0</v>
       </c>
-      <c r="F47" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G47" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="H47" s="7" t="s">
-        <v>116</v>
+      <c r="H47" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I47" s="5" t="s">
         <v>17</v>
@@ -3424,17 +3424,17 @@
         <f t="shared" si="1"/>
         <v>999999953</v>
       </c>
-      <c r="E48" s="5">
+      <c r="E48" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G48" s="5">
         <v>2.0</v>
       </c>
-      <c r="F48" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G48" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="H48" s="7" t="s">
-        <v>118</v>
+      <c r="H48" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="I48" s="5" t="s">
         <v>16</v>
@@ -3463,17 +3463,17 @@
         <f t="shared" si="1"/>
         <v>999999952</v>
       </c>
-      <c r="E49" s="5">
+      <c r="E49" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="G49" s="5">
         <v>3.0</v>
       </c>
-      <c r="F49" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G49" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="H49" s="7" t="s">
-        <v>120</v>
+      <c r="H49" s="5" t="s">
+        <v>31</v>
       </c>
       <c r="I49" s="5" t="s">
         <v>16</v>
@@ -3502,17 +3502,17 @@
         <f t="shared" si="1"/>
         <v>999999951</v>
       </c>
-      <c r="E50" s="5">
+      <c r="E50" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="G50" s="5">
         <v>1.0</v>
       </c>
-      <c r="F50" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G50" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="H50" s="7" t="s">
-        <v>122</v>
+      <c r="H50" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="I50" s="5" t="s">
         <v>22</v>
@@ -3539,17 +3539,17 @@
         <f t="shared" si="1"/>
         <v>999999950</v>
       </c>
-      <c r="E51" s="5">
+      <c r="E51" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="G51" s="5">
         <v>2.0</v>
       </c>
-      <c r="F51" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G51" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="H51" s="7" t="s">
-        <v>124</v>
+      <c r="H51" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="I51" s="5" t="s">
         <v>16</v>
@@ -3572,17 +3572,17 @@
         <f t="shared" si="1"/>
         <v>999999949</v>
       </c>
-      <c r="E52" s="5">
+      <c r="E52" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F52" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="G52" s="5">
         <v>1.0</v>
       </c>
-      <c r="F52" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G52" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="H52" s="13" t="s">
-        <v>126</v>
+      <c r="H52" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I52" s="12" t="s">
         <v>27</v>
@@ -3607,17 +3607,17 @@
         <f t="shared" si="1"/>
         <v>999999948</v>
       </c>
-      <c r="E53" s="5">
+      <c r="E53" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="F53" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="G53" s="5">
         <v>2.0</v>
       </c>
-      <c r="F53" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G53" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="H53" s="13" t="s">
-        <v>128</v>
+      <c r="H53" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I53" s="12" t="s">
         <v>17</v>
@@ -3646,17 +3646,17 @@
         <f t="shared" si="1"/>
         <v>999999947</v>
       </c>
-      <c r="E54" s="5">
+      <c r="E54" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F54" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="G54" s="5">
         <v>3.0</v>
       </c>
-      <c r="F54" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G54" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="H54" s="13" t="s">
-        <v>130</v>
+      <c r="H54" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I54" s="12" t="s">
         <v>16</v>
@@ -3683,17 +3683,17 @@
         <f t="shared" si="1"/>
         <v>999999946</v>
       </c>
-      <c r="E55" s="5">
+      <c r="E55" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="F55" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="G55" s="5">
         <v>1.0</v>
       </c>
-      <c r="F55" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G55" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="H55" s="13" t="s">
-        <v>132</v>
+      <c r="H55" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I55" s="12" t="s">
         <v>22</v>
@@ -3720,17 +3720,17 @@
         <f t="shared" si="1"/>
         <v>999999945</v>
       </c>
-      <c r="E56" s="5">
+      <c r="E56" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="F56" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="G56" s="5">
         <v>2.0</v>
       </c>
-      <c r="F56" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G56" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="H56" s="13" t="s">
-        <v>134</v>
+      <c r="H56" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I56" s="12" t="s">
         <v>22</v>
@@ -3755,17 +3755,17 @@
         <f t="shared" si="1"/>
         <v>999999944</v>
       </c>
-      <c r="E57" s="5">
+      <c r="E57" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="F57" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="G57" s="5">
         <v>3.0</v>
       </c>
-      <c r="F57" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G57" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="H57" s="13" t="s">
-        <v>136</v>
+      <c r="H57" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I57" s="12" t="s">
         <v>16</v>
@@ -3792,17 +3792,17 @@
         <f t="shared" si="1"/>
         <v>999999943</v>
       </c>
-      <c r="E58" s="5">
+      <c r="E58" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="F58" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="G58" s="5">
         <v>1.0</v>
       </c>
-      <c r="F58" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G58" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="H58" s="13" t="s">
-        <v>138</v>
+      <c r="H58" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I58" s="12" t="s">
         <v>22</v>
@@ -3825,17 +3825,17 @@
         <f t="shared" si="1"/>
         <v>999999942</v>
       </c>
-      <c r="E59" s="5">
+      <c r="E59" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="F59" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="G59" s="5">
         <v>2.0</v>
       </c>
-      <c r="F59" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G59" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="H59" s="13" t="s">
-        <v>140</v>
+      <c r="H59" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I59" s="12" t="s">
         <v>16</v>
@@ -3864,17 +3864,17 @@
         <f t="shared" si="1"/>
         <v>999999941</v>
       </c>
-      <c r="E60" s="5">
+      <c r="E60" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="F60" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="G60" s="5">
         <v>3.0</v>
       </c>
-      <c r="F60" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G60" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="H60" s="13" t="s">
-        <v>142</v>
+      <c r="H60" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I60" s="12" t="s">
         <v>16</v>
@@ -3903,17 +3903,17 @@
         <f t="shared" si="1"/>
         <v>999999940</v>
       </c>
-      <c r="E61" s="5">
+      <c r="E61" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="F61" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="G61" s="5">
         <v>1.0</v>
       </c>
-      <c r="F61" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G61" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="H61" s="13" t="s">
-        <v>144</v>
+      <c r="H61" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I61" s="12" t="s">
         <v>22</v>
@@ -3940,17 +3940,17 @@
         <f t="shared" si="1"/>
         <v>999999939</v>
       </c>
-      <c r="E62" s="5">
+      <c r="E62" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="F62" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="G62" s="5">
         <v>2.0</v>
       </c>
-      <c r="F62" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G62" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="H62" s="13" t="s">
-        <v>146</v>
+      <c r="H62" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I62" s="12" t="s">
         <v>22</v>
@@ -3977,17 +3977,17 @@
         <f t="shared" si="1"/>
         <v>999999938</v>
       </c>
-      <c r="E63" s="5">
+      <c r="E63" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="F63" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="G63" s="5">
         <v>3.0</v>
       </c>
-      <c r="F63" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G63" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="H63" s="13" t="s">
-        <v>148</v>
+      <c r="H63" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I63" s="12" t="s">
         <v>22</v>
@@ -4012,17 +4012,17 @@
         <f t="shared" si="1"/>
         <v>999999937</v>
       </c>
-      <c r="E64" s="5">
+      <c r="E64" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="F64" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="G64" s="5">
         <v>1.0</v>
       </c>
-      <c r="F64" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G64" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="H64" s="16" t="s">
-        <v>150</v>
+      <c r="H64" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I64" s="12" t="s">
         <v>17</v>
@@ -4051,17 +4051,17 @@
         <f t="shared" si="1"/>
         <v>999999936</v>
       </c>
-      <c r="E65" s="5">
+      <c r="E65" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="F65" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="G65" s="5">
         <v>2.0</v>
       </c>
-      <c r="F65" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G65" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="H65" s="13" t="s">
-        <v>152</v>
+      <c r="H65" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I65" s="12" t="s">
         <v>22</v>
@@ -4090,17 +4090,17 @@
         <f t="shared" si="1"/>
         <v>999999935</v>
       </c>
-      <c r="E66" s="5">
+      <c r="E66" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="F66" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="G66" s="5">
         <v>3.0</v>
       </c>
-      <c r="F66" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G66" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="H66" s="13" t="s">
-        <v>154</v>
+      <c r="H66" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I66" s="12" t="s">
         <v>16</v>
@@ -4127,17 +4127,17 @@
         <f t="shared" si="1"/>
         <v>999999934</v>
       </c>
-      <c r="E67" s="5">
+      <c r="E67" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="F67" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="G67" s="5">
         <v>1.0</v>
       </c>
-      <c r="F67" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G67" s="12" t="s">
-        <v>156</v>
-      </c>
-      <c r="H67" s="13" t="s">
-        <v>156</v>
+      <c r="H67" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I67" s="12" t="s">
         <v>22</v>
@@ -4160,17 +4160,17 @@
         <f t="shared" si="1"/>
         <v>999999933</v>
       </c>
-      <c r="E68" s="5">
+      <c r="E68" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="F68" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="G68" s="5">
         <v>2.0</v>
       </c>
-      <c r="F68" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G68" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="H68" s="13" t="s">
-        <v>158</v>
+      <c r="H68" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I68" s="12" t="s">
         <v>17</v>
@@ -4199,17 +4199,17 @@
         <f t="shared" si="1"/>
         <v>999999932</v>
       </c>
-      <c r="E69" s="5">
+      <c r="E69" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="F69" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="G69" s="5">
         <v>3.0</v>
       </c>
-      <c r="F69" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G69" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="H69" s="13" t="s">
-        <v>160</v>
+      <c r="H69" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I69" s="12" t="s">
         <v>17</v>
@@ -4238,17 +4238,17 @@
         <f t="shared" si="1"/>
         <v>999999931</v>
       </c>
-      <c r="E70" s="5">
+      <c r="E70" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="F70" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="G70" s="5">
         <v>1.0</v>
       </c>
-      <c r="F70" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G70" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="H70" s="13" t="s">
-        <v>162</v>
+      <c r="H70" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I70" s="12" t="s">
         <v>17</v>
@@ -4277,17 +4277,17 @@
         <f t="shared" si="1"/>
         <v>999999930</v>
       </c>
-      <c r="E71" s="5">
+      <c r="E71" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="F71" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="G71" s="5">
         <v>2.0</v>
       </c>
-      <c r="F71" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G71" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="H71" s="13" t="s">
-        <v>164</v>
+      <c r="H71" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I71" s="12" t="s">
         <v>16</v>
@@ -4312,17 +4312,17 @@
         <f t="shared" si="1"/>
         <v>999999929</v>
       </c>
-      <c r="E72" s="5">
+      <c r="E72" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="F72" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="G72" s="5">
         <v>3.0</v>
       </c>
-      <c r="F72" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G72" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="H72" s="13" t="s">
-        <v>166</v>
+      <c r="H72" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I72" s="12" t="s">
         <v>17</v>
@@ -4349,17 +4349,17 @@
         <f t="shared" si="1"/>
         <v>999999928</v>
       </c>
-      <c r="E73" s="5">
+      <c r="E73" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="F73" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="G73" s="5">
         <v>1.0</v>
       </c>
-      <c r="F73" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G73" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="H73" s="13" t="s">
-        <v>168</v>
+      <c r="H73" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I73" s="12" t="s">
         <v>17</v>
@@ -4386,17 +4386,17 @@
         <f t="shared" si="1"/>
         <v>999999927</v>
       </c>
-      <c r="E74" s="5">
+      <c r="E74" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="F74" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="G74" s="5">
         <v>2.0</v>
       </c>
-      <c r="F74" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G74" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="H74" s="13" t="s">
-        <v>170</v>
+      <c r="H74" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I74" s="12" t="s">
         <v>22</v>
@@ -4419,17 +4419,17 @@
         <f t="shared" si="1"/>
         <v>999999926</v>
       </c>
-      <c r="E75" s="5">
+      <c r="E75" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="F75" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="G75" s="5">
         <v>3.0</v>
       </c>
-      <c r="F75" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G75" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="H75" s="13" t="s">
-        <v>172</v>
+      <c r="H75" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I75" s="12" t="s">
         <v>16</v>
@@ -4458,17 +4458,17 @@
         <f t="shared" si="1"/>
         <v>999999925</v>
       </c>
-      <c r="E76" s="5">
+      <c r="E76" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="F76" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="G76" s="5">
         <v>1.0</v>
       </c>
-      <c r="F76" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G76" s="12" t="s">
-        <v>174</v>
-      </c>
-      <c r="H76" s="13" t="s">
-        <v>174</v>
+      <c r="H76" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I76" s="12" t="s">
         <v>17</v>
@@ -4497,17 +4497,17 @@
         <f t="shared" si="1"/>
         <v>999999924</v>
       </c>
-      <c r="E77" s="5">
+      <c r="E77" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="F77" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="G77" s="5">
         <v>2.0</v>
       </c>
-      <c r="F77" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G77" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="H77" s="13" t="s">
-        <v>176</v>
+      <c r="H77" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I77" s="12" t="s">
         <v>16</v>
@@ -4536,17 +4536,17 @@
         <f t="shared" si="1"/>
         <v>999999923</v>
       </c>
-      <c r="E78" s="5">
+      <c r="E78" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="F78" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="G78" s="5">
         <v>3.0</v>
       </c>
-      <c r="F78" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G78" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="H78" s="13" t="s">
-        <v>178</v>
+      <c r="H78" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I78" s="12" t="s">
         <v>17</v>
@@ -4575,17 +4575,17 @@
         <f t="shared" si="1"/>
         <v>999999922</v>
       </c>
-      <c r="E79" s="5">
+      <c r="E79" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="F79" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="G79" s="5">
         <v>1.0</v>
       </c>
-      <c r="F79" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G79" s="12" t="s">
-        <v>180</v>
-      </c>
-      <c r="H79" s="13" t="s">
-        <v>180</v>
+      <c r="H79" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I79" s="12" t="s">
         <v>16</v>
@@ -4614,17 +4614,17 @@
         <f t="shared" si="1"/>
         <v>999999921</v>
       </c>
-      <c r="E80" s="5">
+      <c r="E80" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="F80" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="G80" s="5">
         <v>2.0</v>
       </c>
-      <c r="F80" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G80" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="H80" s="13" t="s">
-        <v>182</v>
+      <c r="H80" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I80" s="12" t="s">
         <v>22</v>
@@ -4651,17 +4651,17 @@
         <f t="shared" si="1"/>
         <v>999999920</v>
       </c>
-      <c r="E81" s="5">
+      <c r="E81" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="F81" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="G81" s="5">
         <v>3.0</v>
       </c>
-      <c r="F81" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G81" s="12" t="s">
-        <v>184</v>
-      </c>
-      <c r="H81" s="13" t="s">
-        <v>184</v>
+      <c r="H81" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I81" s="12" t="s">
         <v>16</v>
@@ -4688,17 +4688,17 @@
         <f t="shared" si="1"/>
         <v>999999919</v>
       </c>
-      <c r="E82" s="5">
+      <c r="E82" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="F82" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="G82" s="5">
         <v>1.0</v>
       </c>
-      <c r="F82" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G82" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="H82" s="13" t="s">
-        <v>186</v>
+      <c r="H82" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I82" s="12" t="s">
         <v>22</v>
@@ -4727,17 +4727,17 @@
         <f t="shared" si="1"/>
         <v>999999918</v>
       </c>
-      <c r="E83" s="5">
+      <c r="E83" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="F83" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="G83" s="5">
         <v>2.0</v>
       </c>
-      <c r="F83" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G83" s="12" t="s">
-        <v>188</v>
-      </c>
-      <c r="H83" s="13" t="s">
-        <v>188</v>
+      <c r="H83" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I83" s="12" t="s">
         <v>22</v>
@@ -4766,17 +4766,17 @@
         <f t="shared" si="1"/>
         <v>999999917</v>
       </c>
-      <c r="E84" s="5">
+      <c r="E84" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="F84" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="G84" s="5">
         <v>3.0</v>
       </c>
-      <c r="F84" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G84" s="12" t="s">
-        <v>190</v>
-      </c>
-      <c r="H84" s="13" t="s">
-        <v>190</v>
+      <c r="H84" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I84" s="12" t="s">
         <v>22</v>
@@ -4803,17 +4803,17 @@
         <f t="shared" si="1"/>
         <v>999999916</v>
       </c>
-      <c r="E85" s="5">
+      <c r="E85" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="F85" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="G85" s="5">
         <v>1.0</v>
       </c>
-      <c r="F85" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G85" s="12" t="s">
-        <v>192</v>
-      </c>
-      <c r="H85" s="13" t="s">
-        <v>192</v>
+      <c r="H85" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I85" s="12" t="s">
         <v>22</v>
@@ -4842,17 +4842,17 @@
         <f t="shared" si="1"/>
         <v>999999915</v>
       </c>
-      <c r="E86" s="5">
+      <c r="E86" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="F86" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="G86" s="5">
         <v>2.0</v>
       </c>
-      <c r="F86" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G86" s="12" t="s">
-        <v>194</v>
-      </c>
-      <c r="H86" s="13" t="s">
-        <v>194</v>
+      <c r="H86" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I86" s="12" t="s">
         <v>16</v>
@@ -4881,17 +4881,17 @@
         <f t="shared" si="1"/>
         <v>999999914</v>
       </c>
-      <c r="E87" s="5">
+      <c r="E87" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="F87" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="G87" s="5">
         <v>3.0</v>
       </c>
-      <c r="F87" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G87" s="12" t="s">
-        <v>196</v>
-      </c>
-      <c r="H87" s="13" t="s">
-        <v>196</v>
+      <c r="H87" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I87" s="12" t="s">
         <v>22</v>
@@ -4918,17 +4918,17 @@
         <f t="shared" si="1"/>
         <v>999999913</v>
       </c>
-      <c r="E88" s="5">
+      <c r="E88" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="F88" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="G88" s="5">
         <v>1.0</v>
       </c>
-      <c r="F88" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G88" s="12" t="s">
-        <v>198</v>
-      </c>
-      <c r="H88" s="13" t="s">
-        <v>198</v>
+      <c r="H88" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I88" s="12" t="s">
         <v>16</v>
@@ -4957,17 +4957,17 @@
         <f t="shared" si="1"/>
         <v>999999912</v>
       </c>
-      <c r="E89" s="5">
+      <c r="E89" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="F89" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="G89" s="5">
         <v>2.0</v>
       </c>
-      <c r="F89" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G89" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="H89" s="13" t="s">
-        <v>200</v>
+      <c r="H89" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I89" s="12" t="s">
         <v>22</v>
@@ -4994,17 +4994,17 @@
         <f t="shared" si="1"/>
         <v>999999911</v>
       </c>
-      <c r="E90" s="5">
+      <c r="E90" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="F90" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="G90" s="5">
         <v>3.0</v>
       </c>
-      <c r="F90" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G90" s="12" t="s">
-        <v>202</v>
-      </c>
-      <c r="H90" s="13" t="s">
-        <v>202</v>
+      <c r="H90" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I90" s="12" t="s">
         <v>16</v>
@@ -5033,17 +5033,17 @@
         <f t="shared" si="1"/>
         <v>999999910</v>
       </c>
-      <c r="E91" s="5">
+      <c r="E91" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="F91" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="G91" s="5">
         <v>1.0</v>
       </c>
-      <c r="F91" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G91" s="12" t="s">
-        <v>204</v>
-      </c>
-      <c r="H91" s="13" t="s">
-        <v>204</v>
+      <c r="H91" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I91" s="12" t="s">
         <v>22</v>
@@ -5070,17 +5070,17 @@
         <f t="shared" si="1"/>
         <v>999999909</v>
       </c>
-      <c r="E92" s="5">
+      <c r="E92" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="F92" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="G92" s="5">
         <v>2.0</v>
       </c>
-      <c r="F92" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G92" s="12" t="s">
-        <v>206</v>
-      </c>
-      <c r="H92" s="13" t="s">
-        <v>206</v>
+      <c r="H92" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I92" s="12" t="s">
         <v>16</v>
@@ -5103,17 +5103,17 @@
         <f t="shared" si="1"/>
         <v>999999908</v>
       </c>
-      <c r="E93" s="5">
+      <c r="E93" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="F93" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="G93" s="5">
         <v>3.0</v>
       </c>
-      <c r="F93" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G93" s="12" t="s">
-        <v>208</v>
-      </c>
-      <c r="H93" s="13" t="s">
-        <v>208</v>
+      <c r="H93" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I93" s="12" t="s">
         <v>17</v>
@@ -5136,17 +5136,17 @@
         <f t="shared" si="1"/>
         <v>999999907</v>
       </c>
-      <c r="E94" s="5">
+      <c r="E94" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="F94" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="G94" s="5">
         <v>1.0</v>
       </c>
-      <c r="F94" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G94" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="H94" s="13" t="s">
-        <v>210</v>
+      <c r="H94" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I94" s="12" t="s">
         <v>16</v>
@@ -5175,17 +5175,17 @@
         <f t="shared" si="1"/>
         <v>999999906</v>
       </c>
-      <c r="E95" s="5">
+      <c r="E95" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="F95" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="G95" s="5">
         <v>2.0</v>
       </c>
-      <c r="F95" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G95" s="12" t="s">
-        <v>212</v>
-      </c>
-      <c r="H95" s="13" t="s">
-        <v>212</v>
+      <c r="H95" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I95" s="12" t="s">
         <v>16</v>
@@ -5214,17 +5214,17 @@
         <f t="shared" si="1"/>
         <v>999999905</v>
       </c>
-      <c r="E96" s="5">
+      <c r="E96" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="F96" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="G96" s="5">
         <v>3.0</v>
       </c>
-      <c r="F96" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G96" s="12" t="s">
-        <v>214</v>
-      </c>
-      <c r="H96" s="13" t="s">
-        <v>214</v>
+      <c r="H96" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I96" s="12" t="s">
         <v>22</v>
@@ -5253,17 +5253,17 @@
         <f t="shared" si="1"/>
         <v>999999904</v>
       </c>
-      <c r="E97" s="5">
+      <c r="E97" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="F97" s="13" t="s">
+        <v>216</v>
+      </c>
+      <c r="G97" s="5">
         <v>1.0</v>
       </c>
-      <c r="F97" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G97" s="12" t="s">
-        <v>216</v>
-      </c>
-      <c r="H97" s="13" t="s">
-        <v>216</v>
+      <c r="H97" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I97" s="12" t="s">
         <v>22</v>
@@ -5290,17 +5290,17 @@
         <f t="shared" si="1"/>
         <v>999999903</v>
       </c>
-      <c r="E98" s="5">
+      <c r="E98" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="F98" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="G98" s="5">
         <v>2.0</v>
       </c>
-      <c r="F98" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G98" s="12" t="s">
-        <v>218</v>
-      </c>
-      <c r="H98" s="13" t="s">
-        <v>218</v>
+      <c r="H98" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I98" s="12" t="s">
         <v>27</v>
@@ -5323,17 +5323,17 @@
         <f t="shared" si="1"/>
         <v>999999902</v>
       </c>
-      <c r="E99" s="5">
+      <c r="E99" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="F99" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="G99" s="5">
         <v>3.0</v>
       </c>
-      <c r="F99" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G99" s="12" t="s">
-        <v>220</v>
-      </c>
-      <c r="H99" s="13" t="s">
-        <v>220</v>
+      <c r="H99" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I99" s="12" t="s">
         <v>22</v>
@@ -5360,17 +5360,17 @@
         <f t="shared" si="1"/>
         <v>999999901</v>
       </c>
-      <c r="E100" s="5">
+      <c r="E100" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="F100" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="G100" s="5">
         <v>1.0</v>
       </c>
-      <c r="F100" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G100" s="12" t="s">
-        <v>222</v>
-      </c>
-      <c r="H100" s="13" t="s">
-        <v>222</v>
+      <c r="H100" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I100" s="12" t="s">
         <v>22</v>
@@ -5397,17 +5397,17 @@
         <f t="shared" si="1"/>
         <v>999999900</v>
       </c>
-      <c r="E101" s="5">
+      <c r="E101" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="F101" s="13" t="s">
+        <v>224</v>
+      </c>
+      <c r="G101" s="5">
         <v>2.0</v>
       </c>
-      <c r="F101" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G101" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="H101" s="13" t="s">
-        <v>224</v>
+      <c r="H101" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I101" s="12" t="s">
         <v>16</v>
@@ -5434,17 +5434,17 @@
         <f t="shared" si="1"/>
         <v>999999899</v>
       </c>
-      <c r="E102" s="5">
+      <c r="E102" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="F102" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="G102" s="5">
         <v>1.0</v>
       </c>
-      <c r="F102" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G102" s="12" t="s">
-        <v>226</v>
-      </c>
-      <c r="H102" s="13" t="s">
-        <v>226</v>
+      <c r="H102" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I102" s="12" t="s">
         <v>17</v>
@@ -5473,17 +5473,17 @@
         <f t="shared" si="1"/>
         <v>999999898</v>
       </c>
-      <c r="E103" s="5">
+      <c r="E103" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="F103" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="G103" s="5">
         <v>2.0</v>
       </c>
-      <c r="F103" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G103" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="H103" s="13" t="s">
-        <v>228</v>
+      <c r="H103" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I103" s="12" t="s">
         <v>17</v>
@@ -5512,17 +5512,17 @@
         <f t="shared" si="1"/>
         <v>999999897</v>
       </c>
-      <c r="E104" s="5">
+      <c r="E104" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="F104" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="G104" s="5">
         <v>3.0</v>
       </c>
-      <c r="F104" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G104" s="12" t="s">
-        <v>230</v>
-      </c>
-      <c r="H104" s="13" t="s">
-        <v>230</v>
+      <c r="H104" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I104" s="12" t="s">
         <v>16</v>
@@ -5549,17 +5549,17 @@
         <f t="shared" si="1"/>
         <v>999999896</v>
       </c>
-      <c r="E105" s="5">
+      <c r="E105" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="F105" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="G105" s="5">
         <v>1.0</v>
       </c>
-      <c r="F105" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G105" s="12" t="s">
-        <v>232</v>
-      </c>
-      <c r="H105" s="13" t="s">
-        <v>232</v>
+      <c r="H105" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="I105" s="12" t="s">
         <v>22</v>
@@ -5586,17 +5586,17 @@
         <f t="shared" si="1"/>
         <v>999999895</v>
       </c>
-      <c r="E106" s="5">
+      <c r="E106" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="F106" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="G106" s="5">
         <v>2.0</v>
       </c>
-      <c r="F106" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G106" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="H106" s="13" t="s">
-        <v>234</v>
+      <c r="H106" s="12" t="s">
+        <v>15</v>
       </c>
       <c r="I106" s="12" t="s">
         <v>22</v>
@@ -5623,17 +5623,17 @@
         <f t="shared" si="1"/>
         <v>999999894</v>
       </c>
-      <c r="E107" s="5">
+      <c r="E107" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="F107" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="G107" s="5">
         <v>3.0</v>
       </c>
-      <c r="F107" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="G107" s="12" t="s">
-        <v>236</v>
-      </c>
-      <c r="H107" s="13" t="s">
-        <v>236</v>
+      <c r="H107" s="12" t="s">
+        <v>21</v>
       </c>
       <c r="I107" s="12" t="s">
         <v>22</v>
@@ -5656,17 +5656,17 @@
         <f t="shared" si="1"/>
         <v>999999893</v>
       </c>
-      <c r="E108" s="5">
+      <c r="E108" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="F108" s="13" t="s">
+        <v>238</v>
+      </c>
+      <c r="G108" s="5">
         <v>1.0</v>
       </c>
-      <c r="F108" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="G108" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="H108" s="13" t="s">
-        <v>238</v>
+      <c r="H108" s="12" t="s">
+        <v>26</v>
       </c>
       <c r="I108" s="12" t="s">
         <v>22</v>

</xml_diff>